<commit_message>
feat: verify rule CG0428 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000102/negative/01/data/unit-test-coreid-CG0428-negative.xlsx
+++ b/rules/CORE-000102/negative/01/data/unit-test-coreid-CG0428-negative.xlsx
@@ -41,7 +41,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -122,6 +128,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -571,150 +583,150 @@
           <t>PPORRESU</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>PPTOX</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>PPTOXGR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Parameter Short Name</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>Parameter Name</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Result or Finding in Original Units</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>Original Units</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>Toxicity</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>Standard Toxicity Grade</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="n">
+      <c r="E4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="8" t="n">
         <v>50</v>
       </c>
     </row>
@@ -735,12 +747,12 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>TMAX</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Time of CMAX</t>
         </is>
@@ -753,16 +765,12 @@
           <t>h</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>NCI 4.03</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>GRADE 1</t>
-        </is>
-      </c>
+      <c r="J5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -783,20 +791,20 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CMAX</t>
+          <t>TMAX</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Max Conc</t>
+          <t>Time of CMAX</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>44.5</v>
+        <v>1.87</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>ug/L</t>
+          <t>h</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -806,7 +814,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>GRADE 2</t>
+          <t>GRADE 1</t>
         </is>
       </c>
     </row>
@@ -931,7 +939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -963,6 +971,951 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AETERM</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NAUSEA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AETOX</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CTCAE 4.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AETOXGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AETESTCD</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AETEST</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MHTERM</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Fracture</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MHTOX</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>CTCAE 4.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MHTOXGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MHTESTCD</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MHTEST</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CETERM</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Migraine</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CETOX</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CTCAE 4.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CETOXGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CETESTCD</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CETEST</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>eg.xpt</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>EGTESTCD</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>QRSAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>eg.xpt</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>EGTEST</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PR Interval, Aggregate</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>eg.xpt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>EGTOX</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>CTCAE 4.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>eg.xpt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>EGTOXGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>eg.xpt</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>EGTERM</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LBTESTCD</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>HGFR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LBTEST</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Hepatocyte Growth Factor Receptor</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LBTOX</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>CTCAE 4.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LBTOXGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LBTERM</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>pc.xpt</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>PCTESTCD</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>DRUG X</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>6</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>pc.xpt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>5</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>PCTEST</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>STUDYDRUG</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>pc.xpt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>PCTOX</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>NCI 4.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>6</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>pc.xpt</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>5</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>PCTOXGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>6</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>pc.xpt</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>PCTERM</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>pp.xpt</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>PPTESTCD</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>TMAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>7</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>pp.xpt</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>PPTEST</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Time of CMAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>7</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>pp.xpt</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PPTOX</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>NCI 4.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>7</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>pp.xpt</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>5</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>PPTOXGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>7</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>pp.xpt</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>PPTERM</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
         </is>
       </c>
     </row>
@@ -1006,111 +1959,111 @@
           <t>AETERM</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>AETOX</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>AETOXGR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Reported Term for the Adverse Event</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>Toxicity</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Standard Toxicity Grade</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
+      <c r="E4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="8" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1131,17 +2084,17 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>NAUSEA</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>CTCAE 4.03</t>
         </is>
       </c>
-      <c r="G5" s="7" t="n"/>
+      <c r="G5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1162,7 +2115,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>VOMITING</t>
+          <t>NAUSEA</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -1172,7 +2125,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>GRADE 2</t>
+          <t>GRADE 1</t>
         </is>
       </c>
     </row>
@@ -1216,111 +2169,111 @@
           <t>MHTERM</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>MHTOX</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>MHTOXGR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Reported Term for the Medical History</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>Toxicity</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Standard Toxicity Grade</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
+      <c r="E4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="8" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1341,21 +2294,17 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Fracture</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>CTCAE 4.03</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>GRADE 1</t>
-        </is>
-      </c>
+      <c r="G5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1376,7 +2325,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Soft Tissue Damage</t>
+          <t>Fracture</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -1386,7 +2335,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>GRADE 2</t>
+          <t>GRADE 1</t>
         </is>
       </c>
     </row>
@@ -1430,111 +2379,111 @@
           <t>CETERM</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>CETOX</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>CETOXGR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Reported Term for the Clinical Event</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>Toxicity</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Standard Toxicity Grade</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
+      <c r="E4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="8" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1555,21 +2504,17 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Migraine</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>CTCAE 4.03</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>GRADE 1</t>
-        </is>
-      </c>
+      <c r="G5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1590,7 +2535,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Edema</t>
+          <t>Migraine</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -1600,7 +2545,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Char</t>
+          <t>GRADE 1</t>
         </is>
       </c>
     </row>
@@ -1659,150 +2604,150 @@
           <t>EGORRESU</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>EGTOX</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>EGTOXGR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>ECG Test or Examination Short Name</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>ECG Test or Examination Name</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Result or Finding in Original Units</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>Original Units</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>Toxicity</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>Standard Toxicity Grade</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="n">
+      <c r="E4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="8" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1823,12 +2768,12 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>QRSAG</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>PR Interval, Aggregate</t>
         </is>
@@ -1841,12 +2786,12 @@
           <t>sec</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>CTCAE 4.03</t>
         </is>
       </c>
-      <c r="J5" s="7" t="n"/>
+      <c r="J5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1867,20 +2812,20 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>QTAG</t>
+          <t>QRSAG</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>QT Interval, Aggregate</t>
+          <t>PR Interval, Aggregate</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>221</v>
+        <v>0.362</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>msec</t>
+          <t>sec</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -1890,7 +2835,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>GRADE 2</t>
+          <t>GRADE 1</t>
         </is>
       </c>
     </row>
@@ -1949,150 +2894,150 @@
           <t>LBORRESU</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>LBTOX</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>LBTOXGR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Lab Test or Examination Short Name</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>Lab Test or Examination Name</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Result or Finding in Original Units</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>Original Units</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>Toxicity</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>Standard Toxicity Grade</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="n">
+      <c r="E4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="8" t="n">
         <v>50</v>
       </c>
     </row>
@@ -2113,12 +3058,12 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>HGFR</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Hepatocyte Growth Factor Receptor</t>
         </is>
@@ -2131,12 +3076,12 @@
           <t>ng/mL</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>CTCAE 4.03</t>
         </is>
       </c>
-      <c r="J5" s="7" t="n"/>
+      <c r="J5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2157,20 +3102,20 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>GLUC</t>
+          <t>HGFR</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>HGFR</t>
+          <t>Hepatocyte Growth Factor Receptor</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>mg/dL</t>
+          <t>ng/mL</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -2180,7 +3125,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>GRADE 2</t>
+          <t>GRADE 1</t>
         </is>
       </c>
     </row>
@@ -2239,150 +3184,150 @@
           <t>PCORRESU</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>PCTOX</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>PCTOXGR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Pharmacokinetic Test Short Name</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>Pharmacokinetic Test Name</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Result or Finding in Original Units</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>Original Units</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>Toxicity</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>Standard Toxicity Grade</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="A4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="4" t="n">
+      <c r="E4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="8" t="n">
         <v>50</v>
       </c>
     </row>
@@ -2403,12 +3348,12 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>DRUG X</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>STUDYDRUG</t>
         </is>
@@ -2421,16 +3366,12 @@
           <t>ug/mL</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>NCI 4.03</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>GRADE 1</t>
-        </is>
-      </c>
+      <c r="J5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2460,7 +3401,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -2474,7 +3415,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>GRADE 2</t>
+          <t>GRADE 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: remove unwanted output vars and add test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000102/negative/01/data/unit-test-coreid-CG0428-negative.xlsx
+++ b/rules/CORE-000102/negative/01/data/unit-test-coreid-CG0428-negative.xlsx
@@ -747,12 +747,12 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>TMAX</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Time of CMAX</t>
         </is>
@@ -939,7 +939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -993,12 +993,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AETERM</t>
+          <t>AETOX</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>NAUSEA</t>
+          <t>CTCAE 4.03</t>
         </is>
       </c>
     </row>
@@ -1021,22 +1021,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AETOX</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CTCAE 4.03</t>
+          <t>AETOXGR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ae.xpt</t>
+          <t>mh.xpt</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1049,17 +1044,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AETOXGR</t>
+          <t>MHTOX</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CTCAE 4.03</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ae.xpt</t>
+          <t>mh.xpt</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1072,22 +1072,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AETESTCD</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>[ABSENT]</t>
+          <t>MHTOXGR</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ae.xpt</t>
+          <t>ce.xpt</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1100,22 +1095,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AETEST</t>
+          <t>CETOX</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[ABSENT]</t>
+          <t>CTCAE 4.03</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>mh.xpt</t>
+          <t>ce.xpt</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1128,22 +1123,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>MHTERM</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Fracture</t>
+          <t>CETOXGR</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>mh.xpt</t>
+          <t>eg.xpt</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1156,7 +1146,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>MHTOX</t>
+          <t>EGTOX</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1167,11 +1157,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>mh.xpt</t>
+          <t>eg.xpt</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1184,17 +1174,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>MHTOXGR</t>
+          <t>EGTOXGR</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>mh.xpt</t>
+          <t>lb.xpt</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1207,22 +1197,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>MHTESTCD</t>
+          <t>LBTOX</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[ABSENT]</t>
+          <t>CTCAE 4.03</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>mh.xpt</t>
+          <t>lb.xpt</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1235,22 +1225,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MHTEST</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>[ABSENT]</t>
+          <t>LBTOXGR</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ce.xpt</t>
+          <t>pc.xpt</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1263,22 +1248,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CETERM</t>
+          <t>PCTOX</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Migraine</t>
+          <t>NCI 4.03</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ce.xpt</t>
+          <t>pc.xpt</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1291,22 +1276,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CETOX</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>CTCAE 4.03</t>
+          <t>PCTOXGR</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ce.xpt</t>
+          <t>pp.xpt</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1319,17 +1299,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CETOXGR</t>
+          <t>PPTOX</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NCI 4.03</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ce.xpt</t>
+          <t>pp.xpt</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1342,580 +1327,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CETESTCD</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>[ABSENT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>ce.xpt</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>5</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>CETEST</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>[ABSENT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>4</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>eg.xpt</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>5</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>EGTESTCD</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>QRSAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>4</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>eg.xpt</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>5</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>EGTEST</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>PR Interval, Aggregate</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>4</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>eg.xpt</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>5</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>EGTOX</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>CTCAE 4.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>4</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>eg.xpt</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>5</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>EGTOXGR</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>4</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>eg.xpt</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>5</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>EGTERM</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>[ABSENT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>5</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>lb.xpt</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>5</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>LBTESTCD</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>HGFR</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>5</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>lb.xpt</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>5</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>LBTEST</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Hepatocyte Growth Factor Receptor</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>5</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>lb.xpt</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>5</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>LBTOX</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>CTCAE 4.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>5</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>lb.xpt</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>5</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>LBTOXGR</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>5</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>lb.xpt</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>5</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>LBTERM</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>[ABSENT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>6</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>pc.xpt</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>5</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>PCTESTCD</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>DRUG X</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>6</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>pc.xpt</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>5</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>PCTEST</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>STUDYDRUG</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>6</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>pc.xpt</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>5</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>PCTOX</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>NCI 4.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>6</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>pc.xpt</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>5</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>PCTOXGR</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>6</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>pc.xpt</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>5</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>PCTERM</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>[ABSENT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>7</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>pp.xpt</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>5</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>PPTESTCD</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>TMAX</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>7</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>pp.xpt</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>5</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>PPTEST</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Time of CMAX</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>7</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>pp.xpt</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>5</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>PPTOX</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>NCI 4.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>7</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>pp.xpt</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>5</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
           <t>PPTOXGR</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>7</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>pp.xpt</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>5</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>PPTERM</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>[ABSENT]</t>
         </is>
       </c>
     </row>
@@ -2084,7 +1496,7 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>NAUSEA</t>
         </is>
@@ -2294,7 +1706,7 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Fracture</t>
         </is>
@@ -2504,7 +1916,7 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Migraine</t>
         </is>
@@ -2768,12 +2180,12 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>QRSAG</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>PR Interval, Aggregate</t>
         </is>
@@ -3058,12 +2470,12 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>HGFR</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Hepatocyte Growth Factor Receptor</t>
         </is>
@@ -3348,12 +2760,12 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>DRUG X</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>STUDYDRUG</t>
         </is>

</xml_diff>